<commit_message>
Refresh daily regional overview
</commit_message>
<xml_diff>
--- a/pipeline/reports-daily/daily-region-overview.xlsx
+++ b/pipeline/reports-daily/daily-region-overview.xlsx
@@ -645,10 +645,10 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1716</v>
+        <v>1707</v>
       </c>
       <c r="C2" s="7" t="n">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>1107</v>
+        <v>1112</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>85</v>
@@ -671,10 +671,10 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="5">
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>971</v>
+        <v>969</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6">
@@ -697,10 +697,10 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>862</v>
+        <v>858</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7">
@@ -710,10 +710,10 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>767</v>
+        <v>757</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>704</v>
+        <v>709</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>14</v>
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>539</v>
+        <v>548</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>42</v>
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>15</v>
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>6</v>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C14" s="8" t="inlineStr"/>
     </row>
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C15" s="7" t="n">
         <v>11</v>
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C16" s="7" t="n">
         <v>13</v>
@@ -852,7 +852,7 @@
         <v>10000</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>1379</v>
+        <v>1375</v>
       </c>
     </row>
   </sheetData>
@@ -26350,7 +26350,7 @@
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>5 / 1.9 / 0/14</t>
+          <t>3 / 1.8 / 0/14</t>
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr"/>
@@ -26433,7 +26433,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>0 / 0.0 / 0/14</t>
+          <t>1 / 0.1 / 0/14</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
@@ -26681,7 +26681,7 @@
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>4 / 1.1 / 0/14</t>
+          <t>3 / 1.1 / 0/14</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
@@ -26966,7 +26966,7 @@
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>0 / 0.1 / 0/14</t>
+          <t>1 / 0.1 / 0/14</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
@@ -27126,7 +27126,7 @@
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>2 / 2.2 / 0/14</t>
+          <t>1 / 2.1 / 0/14</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
@@ -28085,7 +28085,7 @@
       </c>
       <c r="D51" s="14" t="inlineStr">
         <is>
-          <t>2 / 2.9 / 0/14</t>
+          <t>1 / 2.8 / 0/14</t>
         </is>
       </c>
       <c r="E51" s="14" t="inlineStr">
@@ -28095,7 +28095,7 @@
       </c>
       <c r="F51" s="14" t="inlineStr">
         <is>
-          <t>3 / 1.1 / 0/14</t>
+          <t>2 / 1.1 / 0/14</t>
         </is>
       </c>
       <c r="G51" s="14" t="inlineStr">
@@ -28757,7 +28757,7 @@
       </c>
       <c r="D67" s="14" t="inlineStr">
         <is>
-          <t>1 / 2.6 / 0/14</t>
+          <t>2 / 2.7 / 0/14</t>
         </is>
       </c>
       <c r="E67" s="14" t="inlineStr">
@@ -28809,7 +28809,7 @@
       </c>
       <c r="E68" s="13" t="inlineStr">
         <is>
-          <t>0 / 1.4 / 0/14</t>
+          <t>1 / 1.5 / 0/14</t>
         </is>
       </c>
       <c r="F68" s="13" t="inlineStr">
@@ -28967,7 +28967,7 @@
       <c r="B72" s="13" t="inlineStr"/>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>2 / 1.6 / 0/14</t>
+          <t>1 / 1.5 / 0/14</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
@@ -29075,7 +29075,7 @@
       </c>
       <c r="I74" s="13" t="inlineStr">
         <is>
-          <t>2 / 1.6 / 0/14</t>
+          <t>1 / 1.6 / 0/14</t>
         </is>
       </c>
     </row>
@@ -29113,7 +29113,7 @@
       </c>
       <c r="H75" s="14" t="inlineStr">
         <is>
-          <t>2 / 0.8 / 0/14</t>
+          <t>1 / 0.7 / 0/14</t>
         </is>
       </c>
       <c r="I75" s="14" t="inlineStr">
@@ -29250,7 +29250,7 @@
       <c r="D79" s="14" t="inlineStr"/>
       <c r="E79" s="14" t="inlineStr">
         <is>
-          <t>9 / 5.6 / 5/14</t>
+          <t>11 / 5.7 / 5/14</t>
         </is>
       </c>
       <c r="F79" s="14" t="inlineStr">

</xml_diff>